<commit_message>
docs: align member import template with dapodik date format
</commit_message>
<xml_diff>
--- a/templates/Template_Import_Anggota_v1.0.xlsx
+++ b/templates/Template_Import_Anggota_v1.0.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="63">
   <si>
     <t>Nama</t>
   </si>
@@ -180,16 +180,16 @@
     <t>8.</t>
   </si>
   <si>
-    <t>Tanggal Lahir boleh berupa:</t>
-  </si>
-  <si>
-    <t>tanggal Excel</t>
-  </si>
-  <si>
-    <t>teks tanggal</t>
-  </si>
-  <si>
-    <t>kosong</t>
+    <t>Tanggal Lahir diisi dengan format YYYY-MM-DD.</t>
+  </si>
+  <si>
+    <t>Contoh: 2009-07-27</t>
+  </si>
+  <si>
+    <t>Boleh dikosongkan.</t>
+  </si>
+  <si>
+    <t/>
   </si>
   <si>
     <t>9.</t>
@@ -208,6 +208,12 @@
   </si>
   <si>
     <t>Simpan file dalam format .xlsx.</t>
+  </si>
+  <si>
+    <t>2009-07-27</t>
+  </si>
+  <si>
+    <t>2010-03-15</t>
   </si>
 </sst>
 </file>
@@ -636,8 +642,8 @@
       <c r="E2" t="s">
         <v>13</v>
       </c>
-      <c r="F2" s="3">
-        <v>38949</v>
+      <c r="F2" t="s">
+        <v>61</v>
       </c>
       <c r="G2" t="s">
         <v>14</v>
@@ -665,8 +671,8 @@
       <c r="E3" t="s">
         <v>21</v>
       </c>
-      <c r="F3" s="3">
-        <v>38484</v>
+      <c r="F3" t="s">
+        <v>62</v>
       </c>
       <c r="G3" t="s">
         <v>22</v>
@@ -680,987 +686,987 @@
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D4" s="2"/>
-      <c r="F4" s="3"/>
+      <c r="F4"/>
       <c r="H4" s="2"/>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D5" s="2"/>
-      <c r="F5" s="3"/>
+      <c r="F5"/>
       <c r="H5" s="2"/>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D6" s="2"/>
-      <c r="F6" s="3"/>
+      <c r="F6"/>
       <c r="H6" s="2"/>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D7" s="2"/>
-      <c r="F7" s="3"/>
+      <c r="F7"/>
       <c r="H7" s="2"/>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D8" s="2"/>
-      <c r="F8" s="3"/>
+      <c r="F8"/>
       <c r="H8" s="2"/>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D9" s="2"/>
-      <c r="F9" s="3"/>
+      <c r="F9"/>
       <c r="H9" s="2"/>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D10" s="2"/>
-      <c r="F10" s="3"/>
+      <c r="F10"/>
       <c r="H10" s="2"/>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D11" s="2"/>
-      <c r="F11" s="3"/>
+      <c r="F11"/>
       <c r="H11" s="2"/>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D12" s="2"/>
-      <c r="F12" s="3"/>
+      <c r="F12"/>
       <c r="H12" s="2"/>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D13" s="2"/>
-      <c r="F13" s="3"/>
+      <c r="F13"/>
       <c r="H13" s="2"/>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D14" s="2"/>
-      <c r="F14" s="3"/>
+      <c r="F14"/>
       <c r="H14" s="2"/>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D15" s="2"/>
-      <c r="F15" s="3"/>
+      <c r="F15"/>
       <c r="H15" s="2"/>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D16" s="2"/>
-      <c r="F16" s="3"/>
+      <c r="F16"/>
       <c r="H16" s="2"/>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D17" s="2"/>
-      <c r="F17" s="3"/>
+      <c r="F17"/>
       <c r="H17" s="2"/>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D18" s="2"/>
-      <c r="F18" s="3"/>
+      <c r="F18"/>
       <c r="H18" s="2"/>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D19" s="2"/>
-      <c r="F19" s="3"/>
+      <c r="F19"/>
       <c r="H19" s="2"/>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D20" s="2"/>
-      <c r="F20" s="3"/>
+      <c r="F20"/>
       <c r="H20" s="2"/>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D21" s="2"/>
-      <c r="F21" s="3"/>
+      <c r="F21"/>
       <c r="H21" s="2"/>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D22" s="2"/>
-      <c r="F22" s="3"/>
+      <c r="F22"/>
       <c r="H22" s="2"/>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D23" s="2"/>
-      <c r="F23" s="3"/>
+      <c r="F23"/>
       <c r="H23" s="2"/>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D24" s="2"/>
-      <c r="F24" s="3"/>
+      <c r="F24"/>
       <c r="H24" s="2"/>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D25" s="2"/>
-      <c r="F25" s="3"/>
+      <c r="F25"/>
       <c r="H25" s="2"/>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D26" s="2"/>
-      <c r="F26" s="3"/>
+      <c r="F26"/>
       <c r="H26" s="2"/>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D27" s="2"/>
-      <c r="F27" s="3"/>
+      <c r="F27"/>
       <c r="H27" s="2"/>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D28" s="2"/>
-      <c r="F28" s="3"/>
+      <c r="F28"/>
       <c r="H28" s="2"/>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D29" s="2"/>
-      <c r="F29" s="3"/>
+      <c r="F29"/>
       <c r="H29" s="2"/>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D30" s="2"/>
-      <c r="F30" s="3"/>
+      <c r="F30"/>
       <c r="H30" s="2"/>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D31" s="2"/>
-      <c r="F31" s="3"/>
+      <c r="F31"/>
       <c r="H31" s="2"/>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D32" s="2"/>
-      <c r="F32" s="3"/>
+      <c r="F32"/>
       <c r="H32" s="2"/>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D33" s="2"/>
-      <c r="F33" s="3"/>
+      <c r="F33"/>
       <c r="H33" s="2"/>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D34" s="2"/>
-      <c r="F34" s="3"/>
+      <c r="F34"/>
       <c r="H34" s="2"/>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D35" s="2"/>
-      <c r="F35" s="3"/>
+      <c r="F35"/>
       <c r="H35" s="2"/>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D36" s="2"/>
-      <c r="F36" s="3"/>
+      <c r="F36"/>
       <c r="H36" s="2"/>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D37" s="2"/>
-      <c r="F37" s="3"/>
+      <c r="F37"/>
       <c r="H37" s="2"/>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D38" s="2"/>
-      <c r="F38" s="3"/>
+      <c r="F38"/>
       <c r="H38" s="2"/>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D39" s="2"/>
-      <c r="F39" s="3"/>
+      <c r="F39"/>
       <c r="H39" s="2"/>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D40" s="2"/>
-      <c r="F40" s="3"/>
+      <c r="F40"/>
       <c r="H40" s="2"/>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D41" s="2"/>
-      <c r="F41" s="3"/>
+      <c r="F41"/>
       <c r="H41" s="2"/>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D42" s="2"/>
-      <c r="F42" s="3"/>
+      <c r="F42"/>
       <c r="H42" s="2"/>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D43" s="2"/>
-      <c r="F43" s="3"/>
+      <c r="F43"/>
       <c r="H43" s="2"/>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D44" s="2"/>
-      <c r="F44" s="3"/>
+      <c r="F44"/>
       <c r="H44" s="2"/>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D45" s="2"/>
-      <c r="F45" s="3"/>
+      <c r="F45"/>
       <c r="H45" s="2"/>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D46" s="2"/>
-      <c r="F46" s="3"/>
+      <c r="F46"/>
       <c r="H46" s="2"/>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D47" s="2"/>
-      <c r="F47" s="3"/>
+      <c r="F47"/>
       <c r="H47" s="2"/>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D48" s="2"/>
-      <c r="F48" s="3"/>
+      <c r="F48"/>
       <c r="H48" s="2"/>
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D49" s="2"/>
-      <c r="F49" s="3"/>
+      <c r="F49"/>
       <c r="H49" s="2"/>
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D50" s="2"/>
-      <c r="F50" s="3"/>
+      <c r="F50"/>
       <c r="H50" s="2"/>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D51" s="2"/>
-      <c r="F51" s="3"/>
+      <c r="F51"/>
       <c r="H51" s="2"/>
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D52" s="2"/>
-      <c r="F52" s="3"/>
+      <c r="F52"/>
       <c r="H52" s="2"/>
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D53" s="2"/>
-      <c r="F53" s="3"/>
+      <c r="F53"/>
       <c r="H53" s="2"/>
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D54" s="2"/>
-      <c r="F54" s="3"/>
+      <c r="F54"/>
       <c r="H54" s="2"/>
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D55" s="2"/>
-      <c r="F55" s="3"/>
+      <c r="F55"/>
       <c r="H55" s="2"/>
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D56" s="2"/>
-      <c r="F56" s="3"/>
+      <c r="F56"/>
       <c r="H56" s="2"/>
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D57" s="2"/>
-      <c r="F57" s="3"/>
+      <c r="F57"/>
       <c r="H57" s="2"/>
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D58" s="2"/>
-      <c r="F58" s="3"/>
+      <c r="F58"/>
       <c r="H58" s="2"/>
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D59" s="2"/>
-      <c r="F59" s="3"/>
+      <c r="F59"/>
       <c r="H59" s="2"/>
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D60" s="2"/>
-      <c r="F60" s="3"/>
+      <c r="F60"/>
       <c r="H60" s="2"/>
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D61" s="2"/>
-      <c r="F61" s="3"/>
+      <c r="F61"/>
       <c r="H61" s="2"/>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D62" s="2"/>
-      <c r="F62" s="3"/>
+      <c r="F62"/>
       <c r="H62" s="2"/>
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D63" s="2"/>
-      <c r="F63" s="3"/>
+      <c r="F63"/>
       <c r="H63" s="2"/>
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D64" s="2"/>
-      <c r="F64" s="3"/>
+      <c r="F64"/>
       <c r="H64" s="2"/>
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D65" s="2"/>
-      <c r="F65" s="3"/>
+      <c r="F65"/>
       <c r="H65" s="2"/>
     </row>
     <row r="66" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D66" s="2"/>
-      <c r="F66" s="3"/>
+      <c r="F66"/>
       <c r="H66" s="2"/>
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D67" s="2"/>
-      <c r="F67" s="3"/>
+      <c r="F67"/>
       <c r="H67" s="2"/>
     </row>
     <row r="68" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D68" s="2"/>
-      <c r="F68" s="3"/>
+      <c r="F68"/>
       <c r="H68" s="2"/>
     </row>
     <row r="69" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D69" s="2"/>
-      <c r="F69" s="3"/>
+      <c r="F69"/>
       <c r="H69" s="2"/>
     </row>
     <row r="70" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D70" s="2"/>
-      <c r="F70" s="3"/>
+      <c r="F70"/>
       <c r="H70" s="2"/>
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D71" s="2"/>
-      <c r="F71" s="3"/>
+      <c r="F71"/>
       <c r="H71" s="2"/>
     </row>
     <row r="72" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D72" s="2"/>
-      <c r="F72" s="3"/>
+      <c r="F72"/>
       <c r="H72" s="2"/>
     </row>
     <row r="73" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D73" s="2"/>
-      <c r="F73" s="3"/>
+      <c r="F73"/>
       <c r="H73" s="2"/>
     </row>
     <row r="74" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D74" s="2"/>
-      <c r="F74" s="3"/>
+      <c r="F74"/>
       <c r="H74" s="2"/>
     </row>
     <row r="75" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D75" s="2"/>
-      <c r="F75" s="3"/>
+      <c r="F75"/>
       <c r="H75" s="2"/>
     </row>
     <row r="76" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D76" s="2"/>
-      <c r="F76" s="3"/>
+      <c r="F76"/>
       <c r="H76" s="2"/>
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D77" s="2"/>
-      <c r="F77" s="3"/>
+      <c r="F77"/>
       <c r="H77" s="2"/>
     </row>
     <row r="78" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D78" s="2"/>
-      <c r="F78" s="3"/>
+      <c r="F78"/>
       <c r="H78" s="2"/>
     </row>
     <row r="79" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D79" s="2"/>
-      <c r="F79" s="3"/>
+      <c r="F79"/>
       <c r="H79" s="2"/>
     </row>
     <row r="80" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D80" s="2"/>
-      <c r="F80" s="3"/>
+      <c r="F80"/>
       <c r="H80" s="2"/>
     </row>
     <row r="81" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D81" s="2"/>
-      <c r="F81" s="3"/>
+      <c r="F81"/>
       <c r="H81" s="2"/>
     </row>
     <row r="82" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D82" s="2"/>
-      <c r="F82" s="3"/>
+      <c r="F82"/>
       <c r="H82" s="2"/>
     </row>
     <row r="83" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D83" s="2"/>
-      <c r="F83" s="3"/>
+      <c r="F83"/>
       <c r="H83" s="2"/>
     </row>
     <row r="84" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D84" s="2"/>
-      <c r="F84" s="3"/>
+      <c r="F84"/>
       <c r="H84" s="2"/>
     </row>
     <row r="85" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D85" s="2"/>
-      <c r="F85" s="3"/>
+      <c r="F85"/>
       <c r="H85" s="2"/>
     </row>
     <row r="86" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D86" s="2"/>
-      <c r="F86" s="3"/>
+      <c r="F86"/>
       <c r="H86" s="2"/>
     </row>
     <row r="87" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D87" s="2"/>
-      <c r="F87" s="3"/>
+      <c r="F87"/>
       <c r="H87" s="2"/>
     </row>
     <row r="88" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D88" s="2"/>
-      <c r="F88" s="3"/>
+      <c r="F88"/>
       <c r="H88" s="2"/>
     </row>
     <row r="89" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D89" s="2"/>
-      <c r="F89" s="3"/>
+      <c r="F89"/>
       <c r="H89" s="2"/>
     </row>
     <row r="90" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D90" s="2"/>
-      <c r="F90" s="3"/>
+      <c r="F90"/>
       <c r="H90" s="2"/>
     </row>
     <row r="91" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D91" s="2"/>
-      <c r="F91" s="3"/>
+      <c r="F91"/>
       <c r="H91" s="2"/>
     </row>
     <row r="92" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D92" s="2"/>
-      <c r="F92" s="3"/>
+      <c r="F92"/>
       <c r="H92" s="2"/>
     </row>
     <row r="93" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D93" s="2"/>
-      <c r="F93" s="3"/>
+      <c r="F93"/>
       <c r="H93" s="2"/>
     </row>
     <row r="94" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D94" s="2"/>
-      <c r="F94" s="3"/>
+      <c r="F94"/>
       <c r="H94" s="2"/>
     </row>
     <row r="95" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D95" s="2"/>
-      <c r="F95" s="3"/>
+      <c r="F95"/>
       <c r="H95" s="2"/>
     </row>
     <row r="96" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D96" s="2"/>
-      <c r="F96" s="3"/>
+      <c r="F96"/>
       <c r="H96" s="2"/>
     </row>
     <row r="97" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D97" s="2"/>
-      <c r="F97" s="3"/>
+      <c r="F97"/>
       <c r="H97" s="2"/>
     </row>
     <row r="98" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D98" s="2"/>
-      <c r="F98" s="3"/>
+      <c r="F98"/>
       <c r="H98" s="2"/>
     </row>
     <row r="99" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D99" s="2"/>
-      <c r="F99" s="3"/>
+      <c r="F99"/>
       <c r="H99" s="2"/>
     </row>
     <row r="100" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D100" s="2"/>
-      <c r="F100" s="3"/>
+      <c r="F100"/>
       <c r="H100" s="2"/>
     </row>
     <row r="101" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D101" s="2"/>
-      <c r="F101" s="3"/>
+      <c r="F101"/>
       <c r="H101" s="2"/>
     </row>
     <row r="102" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D102" s="2"/>
-      <c r="F102" s="3"/>
+      <c r="F102"/>
       <c r="H102" s="2"/>
     </row>
     <row r="103" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D103" s="2"/>
-      <c r="F103" s="3"/>
+      <c r="F103"/>
       <c r="H103" s="2"/>
     </row>
     <row r="104" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D104" s="2"/>
-      <c r="F104" s="3"/>
+      <c r="F104"/>
       <c r="H104" s="2"/>
     </row>
     <row r="105" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D105" s="2"/>
-      <c r="F105" s="3"/>
+      <c r="F105"/>
       <c r="H105" s="2"/>
     </row>
     <row r="106" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D106" s="2"/>
-      <c r="F106" s="3"/>
+      <c r="F106"/>
       <c r="H106" s="2"/>
     </row>
     <row r="107" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D107" s="2"/>
-      <c r="F107" s="3"/>
+      <c r="F107"/>
       <c r="H107" s="2"/>
     </row>
     <row r="108" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D108" s="2"/>
-      <c r="F108" s="3"/>
+      <c r="F108"/>
       <c r="H108" s="2"/>
     </row>
     <row r="109" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D109" s="2"/>
-      <c r="F109" s="3"/>
+      <c r="F109"/>
       <c r="H109" s="2"/>
     </row>
     <row r="110" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D110" s="2"/>
-      <c r="F110" s="3"/>
+      <c r="F110"/>
       <c r="H110" s="2"/>
     </row>
     <row r="111" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D111" s="2"/>
-      <c r="F111" s="3"/>
+      <c r="F111"/>
       <c r="H111" s="2"/>
     </row>
     <row r="112" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D112" s="2"/>
-      <c r="F112" s="3"/>
+      <c r="F112"/>
       <c r="H112" s="2"/>
     </row>
     <row r="113" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D113" s="2"/>
-      <c r="F113" s="3"/>
+      <c r="F113"/>
       <c r="H113" s="2"/>
     </row>
     <row r="114" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D114" s="2"/>
-      <c r="F114" s="3"/>
+      <c r="F114"/>
       <c r="H114" s="2"/>
     </row>
     <row r="115" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D115" s="2"/>
-      <c r="F115" s="3"/>
+      <c r="F115"/>
       <c r="H115" s="2"/>
     </row>
     <row r="116" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D116" s="2"/>
-      <c r="F116" s="3"/>
+      <c r="F116"/>
       <c r="H116" s="2"/>
     </row>
     <row r="117" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D117" s="2"/>
-      <c r="F117" s="3"/>
+      <c r="F117"/>
       <c r="H117" s="2"/>
     </row>
     <row r="118" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D118" s="2"/>
-      <c r="F118" s="3"/>
+      <c r="F118"/>
       <c r="H118" s="2"/>
     </row>
     <row r="119" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D119" s="2"/>
-      <c r="F119" s="3"/>
+      <c r="F119"/>
       <c r="H119" s="2"/>
     </row>
     <row r="120" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D120" s="2"/>
-      <c r="F120" s="3"/>
+      <c r="F120"/>
       <c r="H120" s="2"/>
     </row>
     <row r="121" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D121" s="2"/>
-      <c r="F121" s="3"/>
+      <c r="F121"/>
       <c r="H121" s="2"/>
     </row>
     <row r="122" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D122" s="2"/>
-      <c r="F122" s="3"/>
+      <c r="F122"/>
       <c r="H122" s="2"/>
     </row>
     <row r="123" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D123" s="2"/>
-      <c r="F123" s="3"/>
+      <c r="F123"/>
       <c r="H123" s="2"/>
     </row>
     <row r="124" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D124" s="2"/>
-      <c r="F124" s="3"/>
+      <c r="F124"/>
       <c r="H124" s="2"/>
     </row>
     <row r="125" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D125" s="2"/>
-      <c r="F125" s="3"/>
+      <c r="F125"/>
       <c r="H125" s="2"/>
     </row>
     <row r="126" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D126" s="2"/>
-      <c r="F126" s="3"/>
+      <c r="F126"/>
       <c r="H126" s="2"/>
     </row>
     <row r="127" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D127" s="2"/>
-      <c r="F127" s="3"/>
+      <c r="F127"/>
       <c r="H127" s="2"/>
     </row>
     <row r="128" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D128" s="2"/>
-      <c r="F128" s="3"/>
+      <c r="F128"/>
       <c r="H128" s="2"/>
     </row>
     <row r="129" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D129" s="2"/>
-      <c r="F129" s="3"/>
+      <c r="F129"/>
       <c r="H129" s="2"/>
     </row>
     <row r="130" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D130" s="2"/>
-      <c r="F130" s="3"/>
+      <c r="F130"/>
       <c r="H130" s="2"/>
     </row>
     <row r="131" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D131" s="2"/>
-      <c r="F131" s="3"/>
+      <c r="F131"/>
       <c r="H131" s="2"/>
     </row>
     <row r="132" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D132" s="2"/>
-      <c r="F132" s="3"/>
+      <c r="F132"/>
       <c r="H132" s="2"/>
     </row>
     <row r="133" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D133" s="2"/>
-      <c r="F133" s="3"/>
+      <c r="F133"/>
       <c r="H133" s="2"/>
     </row>
     <row r="134" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D134" s="2"/>
-      <c r="F134" s="3"/>
+      <c r="F134"/>
       <c r="H134" s="2"/>
     </row>
     <row r="135" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D135" s="2"/>
-      <c r="F135" s="3"/>
+      <c r="F135"/>
       <c r="H135" s="2"/>
     </row>
     <row r="136" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D136" s="2"/>
-      <c r="F136" s="3"/>
+      <c r="F136"/>
       <c r="H136" s="2"/>
     </row>
     <row r="137" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D137" s="2"/>
-      <c r="F137" s="3"/>
+      <c r="F137"/>
       <c r="H137" s="2"/>
     </row>
     <row r="138" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D138" s="2"/>
-      <c r="F138" s="3"/>
+      <c r="F138"/>
       <c r="H138" s="2"/>
     </row>
     <row r="139" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D139" s="2"/>
-      <c r="F139" s="3"/>
+      <c r="F139"/>
       <c r="H139" s="2"/>
     </row>
     <row r="140" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D140" s="2"/>
-      <c r="F140" s="3"/>
+      <c r="F140"/>
       <c r="H140" s="2"/>
     </row>
     <row r="141" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D141" s="2"/>
-      <c r="F141" s="3"/>
+      <c r="F141"/>
       <c r="H141" s="2"/>
     </row>
     <row r="142" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D142" s="2"/>
-      <c r="F142" s="3"/>
+      <c r="F142"/>
       <c r="H142" s="2"/>
     </row>
     <row r="143" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D143" s="2"/>
-      <c r="F143" s="3"/>
+      <c r="F143"/>
       <c r="H143" s="2"/>
     </row>
     <row r="144" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D144" s="2"/>
-      <c r="F144" s="3"/>
+      <c r="F144"/>
       <c r="H144" s="2"/>
     </row>
     <row r="145" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D145" s="2"/>
-      <c r="F145" s="3"/>
+      <c r="F145"/>
       <c r="H145" s="2"/>
     </row>
     <row r="146" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D146" s="2"/>
-      <c r="F146" s="3"/>
+      <c r="F146"/>
       <c r="H146" s="2"/>
     </row>
     <row r="147" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D147" s="2"/>
-      <c r="F147" s="3"/>
+      <c r="F147"/>
       <c r="H147" s="2"/>
     </row>
     <row r="148" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D148" s="2"/>
-      <c r="F148" s="3"/>
+      <c r="F148"/>
       <c r="H148" s="2"/>
     </row>
     <row r="149" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D149" s="2"/>
-      <c r="F149" s="3"/>
+      <c r="F149"/>
       <c r="H149" s="2"/>
     </row>
     <row r="150" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D150" s="2"/>
-      <c r="F150" s="3"/>
+      <c r="F150"/>
       <c r="H150" s="2"/>
     </row>
     <row r="151" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D151" s="2"/>
-      <c r="F151" s="3"/>
+      <c r="F151"/>
       <c r="H151" s="2"/>
     </row>
     <row r="152" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D152" s="2"/>
-      <c r="F152" s="3"/>
+      <c r="F152"/>
       <c r="H152" s="2"/>
     </row>
     <row r="153" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D153" s="2"/>
-      <c r="F153" s="3"/>
+      <c r="F153"/>
       <c r="H153" s="2"/>
     </row>
     <row r="154" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D154" s="2"/>
-      <c r="F154" s="3"/>
+      <c r="F154"/>
       <c r="H154" s="2"/>
     </row>
     <row r="155" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D155" s="2"/>
-      <c r="F155" s="3"/>
+      <c r="F155"/>
       <c r="H155" s="2"/>
     </row>
     <row r="156" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D156" s="2"/>
-      <c r="F156" s="3"/>
+      <c r="F156"/>
       <c r="H156" s="2"/>
     </row>
     <row r="157" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D157" s="2"/>
-      <c r="F157" s="3"/>
+      <c r="F157"/>
       <c r="H157" s="2"/>
     </row>
     <row r="158" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D158" s="2"/>
-      <c r="F158" s="3"/>
+      <c r="F158"/>
       <c r="H158" s="2"/>
     </row>
     <row r="159" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D159" s="2"/>
-      <c r="F159" s="3"/>
+      <c r="F159"/>
       <c r="H159" s="2"/>
     </row>
     <row r="160" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D160" s="2"/>
-      <c r="F160" s="3"/>
+      <c r="F160"/>
       <c r="H160" s="2"/>
     </row>
     <row r="161" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D161" s="2"/>
-      <c r="F161" s="3"/>
+      <c r="F161"/>
       <c r="H161" s="2"/>
     </row>
     <row r="162" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D162" s="2"/>
-      <c r="F162" s="3"/>
+      <c r="F162"/>
       <c r="H162" s="2"/>
     </row>
     <row r="163" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D163" s="2"/>
-      <c r="F163" s="3"/>
+      <c r="F163"/>
       <c r="H163" s="2"/>
     </row>
     <row r="164" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D164" s="2"/>
-      <c r="F164" s="3"/>
+      <c r="F164"/>
       <c r="H164" s="2"/>
     </row>
     <row r="165" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D165" s="2"/>
-      <c r="F165" s="3"/>
+      <c r="F165"/>
       <c r="H165" s="2"/>
     </row>
     <row r="166" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D166" s="2"/>
-      <c r="F166" s="3"/>
+      <c r="F166"/>
       <c r="H166" s="2"/>
     </row>
     <row r="167" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D167" s="2"/>
-      <c r="F167" s="3"/>
+      <c r="F167"/>
       <c r="H167" s="2"/>
     </row>
     <row r="168" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D168" s="2"/>
-      <c r="F168" s="3"/>
+      <c r="F168"/>
       <c r="H168" s="2"/>
     </row>
     <row r="169" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D169" s="2"/>
-      <c r="F169" s="3"/>
+      <c r="F169"/>
       <c r="H169" s="2"/>
     </row>
     <row r="170" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D170" s="2"/>
-      <c r="F170" s="3"/>
+      <c r="F170"/>
       <c r="H170" s="2"/>
     </row>
     <row r="171" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D171" s="2"/>
-      <c r="F171" s="3"/>
+      <c r="F171"/>
       <c r="H171" s="2"/>
     </row>
     <row r="172" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D172" s="2"/>
-      <c r="F172" s="3"/>
+      <c r="F172"/>
       <c r="H172" s="2"/>
     </row>
     <row r="173" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D173" s="2"/>
-      <c r="F173" s="3"/>
+      <c r="F173"/>
       <c r="H173" s="2"/>
     </row>
     <row r="174" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D174" s="2"/>
-      <c r="F174" s="3"/>
+      <c r="F174"/>
       <c r="H174" s="2"/>
     </row>
     <row r="175" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D175" s="2"/>
-      <c r="F175" s="3"/>
+      <c r="F175"/>
       <c r="H175" s="2"/>
     </row>
     <row r="176" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D176" s="2"/>
-      <c r="F176" s="3"/>
+      <c r="F176"/>
       <c r="H176" s="2"/>
     </row>
     <row r="177" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D177" s="2"/>
-      <c r="F177" s="3"/>
+      <c r="F177"/>
       <c r="H177" s="2"/>
     </row>
     <row r="178" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D178" s="2"/>
-      <c r="F178" s="3"/>
+      <c r="F178"/>
       <c r="H178" s="2"/>
     </row>
     <row r="179" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D179" s="2"/>
-      <c r="F179" s="3"/>
+      <c r="F179"/>
       <c r="H179" s="2"/>
     </row>
     <row r="180" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D180" s="2"/>
-      <c r="F180" s="3"/>
+      <c r="F180"/>
       <c r="H180" s="2"/>
     </row>
     <row r="181" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D181" s="2"/>
-      <c r="F181" s="3"/>
+      <c r="F181"/>
       <c r="H181" s="2"/>
     </row>
     <row r="182" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D182" s="2"/>
-      <c r="F182" s="3"/>
+      <c r="F182"/>
       <c r="H182" s="2"/>
     </row>
     <row r="183" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D183" s="2"/>
-      <c r="F183" s="3"/>
+      <c r="F183"/>
       <c r="H183" s="2"/>
     </row>
     <row r="184" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D184" s="2"/>
-      <c r="F184" s="3"/>
+      <c r="F184"/>
       <c r="H184" s="2"/>
     </row>
     <row r="185" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D185" s="2"/>
-      <c r="F185" s="3"/>
+      <c r="F185"/>
       <c r="H185" s="2"/>
     </row>
     <row r="186" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D186" s="2"/>
-      <c r="F186" s="3"/>
+      <c r="F186"/>
       <c r="H186" s="2"/>
     </row>
     <row r="187" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D187" s="2"/>
-      <c r="F187" s="3"/>
+      <c r="F187"/>
       <c r="H187" s="2"/>
     </row>
     <row r="188" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D188" s="2"/>
-      <c r="F188" s="3"/>
+      <c r="F188"/>
       <c r="H188" s="2"/>
     </row>
     <row r="189" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D189" s="2"/>
-      <c r="F189" s="3"/>
+      <c r="F189"/>
       <c r="H189" s="2"/>
     </row>
     <row r="190" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D190" s="2"/>
-      <c r="F190" s="3"/>
+      <c r="F190"/>
       <c r="H190" s="2"/>
     </row>
     <row r="191" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D191" s="2"/>
-      <c r="F191" s="3"/>
+      <c r="F191"/>
       <c r="H191" s="2"/>
     </row>
     <row r="192" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D192" s="2"/>
-      <c r="F192" s="3"/>
+      <c r="F192"/>
       <c r="H192" s="2"/>
     </row>
     <row r="193" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D193" s="2"/>
-      <c r="F193" s="3"/>
+      <c r="F193"/>
       <c r="H193" s="2"/>
     </row>
     <row r="194" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D194" s="2"/>
-      <c r="F194" s="3"/>
+      <c r="F194"/>
       <c r="H194" s="2"/>
     </row>
     <row r="195" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D195" s="2"/>
-      <c r="F195" s="3"/>
+      <c r="F195"/>
       <c r="H195" s="2"/>
     </row>
     <row r="196" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D196" s="2"/>
-      <c r="F196" s="3"/>
+      <c r="F196"/>
       <c r="H196" s="2"/>
     </row>
     <row r="197" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D197" s="2"/>
-      <c r="F197" s="3"/>
+      <c r="F197"/>
       <c r="H197" s="2"/>
     </row>
     <row r="198" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D198" s="2"/>
-      <c r="F198" s="3"/>
+      <c r="F198"/>
       <c r="H198" s="2"/>
     </row>
     <row r="199" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D199" s="2"/>
-      <c r="F199" s="3"/>
+      <c r="F199"/>
       <c r="H199" s="2"/>
     </row>
     <row r="200" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D200" s="2"/>
-      <c r="F200" s="3"/>
+      <c r="F200"/>
       <c r="H200" s="2"/>
     </row>
   </sheetData>
@@ -1670,5 +1676,5 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="UTF-8" standalone="yes"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"><dimension ref="A1:B35"/><sheetFormatPr defaultRowHeight="15"/><cols><col min="1" max="1" width="8" customWidth="1"/><col min="2" max="2" width="100" customWidth="1"/></cols><sheetData><row r="1" spans="1:2" x14ac:dyDescent="0.25"><c r="A1" s="6" t="s"><v>25</v></c></row><row r="2" spans="1:2" x14ac:dyDescent="0.25"><c r="A2" s="7" t="s"><v>26</v></c></row><row r="3" spans="1:2" x14ac:dyDescent="0.25"><c r="A3" s="7" t="s"><v>28</v></c><c r="B3" s="7" t="s"><v>29</v></c></row><row r="4" spans="1:2" x14ac:dyDescent="0.25"><c r="A4" s="7" t="s"><v>30</v></c><c r="B4" s="7" t="s"><v>31</v></c></row><row r="5" spans="1:2" x14ac:dyDescent="0.25"><c r="A5" s="7" t="s"><v>27</v></c><c r="B5" s="7" t="s"><v>0</v></c></row><row r="6" spans="1:2" x14ac:dyDescent="0.25"><c r="A6" s="7" t="s"><v>27</v></c><c r="B6" s="7" t="s"><v>1</v></c></row><row r="7" spans="1:2" x14ac:dyDescent="0.25"><c r="A7" s="7" t="s"><v>27</v></c><c r="B7" s="7" t="s"><v>2</v></c></row><row r="8" spans="1:2" x14ac:dyDescent="0.25"><c r="A8" s="7" t="s"><v>27</v></c><c r="B8" s="7" t="s"><v>3</v></c></row><row r="9" spans="1:2" x14ac:dyDescent="0.25"><c r="A9" s="7" t="s"><v>27</v></c><c r="B9" s="7" t="s"><v>6</v></c></row><row r="10" spans="1:2" x14ac:dyDescent="0.25"><c r="A10" s="7" t="s"><v>27</v></c><c r="B10" s="7" t="s"><v>7</v></c></row><row r="11" spans="1:2" x14ac:dyDescent="0.25"><c r="A11" s="7" t="s"><v>32</v></c><c r="B11" s="7" t="s"><v>33</v></c></row><row r="12" spans="1:2" x14ac:dyDescent="0.25"><c r="A12" s="7" t="s"><v>27</v></c><c r="B12" s="7" t="s"><v>4</v></c></row><row r="13" spans="1:2" x14ac:dyDescent="0.25"><c r="A13" s="7" t="s"><v>27</v></c><c r="B13" s="7" t="s"><v>5</v></c></row><row r="14" spans="1:2" x14ac:dyDescent="0.25"><c r="A14" s="7" t="s"><v>27</v></c><c r="B14" s="7" t="s"><v>8</v></c></row><row r="15" spans="1:2" x14ac:dyDescent="0.25"><c r="A15" s="7" t="s"><v>34</v></c><c r="B15" s="7" t="s"><v>35</v></c></row><row r="16" spans="1:2" x14ac:dyDescent="0.25"><c r="A16" s="7" t="s"><v>36</v></c><c r="B16" s="7" t="s"><v>37</v></c></row><row r="17" spans="1:2" x14ac:dyDescent="0.25"><c r="A17" s="7" t="s"><v>38</v></c><c r="B17" s="7" t="s"><v>39</v></c></row><row r="18" spans="1:2" x14ac:dyDescent="0.25"><c r="A18" s="7" t="s"><v>27</v></c><c r="B18" s="7" t="s"><v>40</v></c></row><row r="19" spans="1:2" x14ac:dyDescent="0.25"><c r="A19" s="7" t="s"><v>27</v></c><c r="B19" s="7" t="s"><v>41</v></c></row><row r="20" spans="1:2" x14ac:dyDescent="0.25"><c r="A20" s="7" t="s"><v>27</v></c><c r="B20" s="7" t="s"><v>42</v></c></row><row r="21" spans="1:2" x14ac:dyDescent="0.25"><c r="A21" s="7" t="s"><v>27</v></c><c r="B21" s="7" t="s"><v>43</v></c></row><row r="22" spans="1:2" x14ac:dyDescent="0.25"><c r="A22" s="7" t="s"><v>27</v></c><c r="B22" s="7" t="s"><v>44</v></c></row><row r="23" spans="1:2" x14ac:dyDescent="0.25"><c r="A23" s="7" t="s"><v>27</v></c><c r="B23" s="7" t="s"><v>45</v></c></row><row r="24" spans="1:2" x14ac:dyDescent="0.25"><c r="A24" s="7" t="s"><v>46</v></c><c r="B24" s="7" t="s"><v>47</v></c></row><row r="25" spans="1:2" x14ac:dyDescent="0.25"><c r="A25" s="7" t="s"><v>27</v></c><c r="B25" s="7" t="s"><v>11</v></c></row><row r="26" spans="1:2" x14ac:dyDescent="0.25"><c r="A26" s="7" t="s"><v>27</v></c><c r="B26" s="7" t="s"><v>48</v></c></row><row r="27" spans="1:2" x14ac:dyDescent="0.25"><c r="A27" s="7" t="s"><v>27</v></c><c r="B27" s="7" t="s"><v>19</v></c></row><row r="28" spans="1:2" x14ac:dyDescent="0.25"><c r="A28" s="7" t="s"><v>27</v></c><c r="B28" s="7" t="s"><v>49</v></c></row><row r="29" spans="1:2" x14ac:dyDescent="0.25"><c r="A29" s="7" t="s"><v>50</v></c><c r="B29" s="7" t="s"><v>51</v></c></row><row r="30" spans="1:2" x14ac:dyDescent="0.25"><c r="A30" s="7" t="s"><v>27</v></c><c r="B30" s="7" t="s"><v>52</v></c></row><row r="31" spans="1:2" x14ac:dyDescent="0.25"><c r="A31" s="7" t="s"><v>27</v></c><c r="B31" s="7" t="s"><v>53</v></c></row><row r="32" spans="1:2" x14ac:dyDescent="0.25"><c r="A32" s="7" t="s"><v>27</v></c><c r="B32" s="7" t="s"><v>54</v></c></row><row r="33" spans="1:2" x14ac:dyDescent="0.25"><c r="A33" s="7" t="s"><v>55</v></c><c r="B33" s="7" t="s"><v>56</v></c></row><row r="34" spans="1:2" x14ac:dyDescent="0.25"><c r="A34" s="7" t="s"><v>57</v></c><c r="B34" s="7" t="s"><v>58</v></c></row><row r="35" spans="1:2" x14ac:dyDescent="0.25"><c r="A35" s="7" t="s"><v>59</v></c><c r="B35" s="7" t="s"><v>60</v></c></row></sheetData><mergeCells count="2"><mergeCell ref="A1:B1"/><mergeCell ref="A2:B2"/></mergeCells><pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/></worksheet>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"><dimension ref="A1:B35"/><sheetFormatPr defaultRowHeight="15"/><cols><col min="1" max="1" width="8" customWidth="1"/><col min="2" max="2" width="100" customWidth="1"/></cols><sheetData><row r="1" spans="1:2" x14ac:dyDescent="0.25"><c r="A1" s="6" t="s"><v>25</v></c></row><row r="2" spans="1:2" x14ac:dyDescent="0.25"><c r="A2" s="7" t="s"><v>26</v></c></row><row r="3" spans="1:2" x14ac:dyDescent="0.25"><c r="A3" s="7" t="s"><v>28</v></c><c r="B3" s="7" t="s"><v>29</v></c></row><row r="4" spans="1:2" x14ac:dyDescent="0.25"><c r="A4" s="7" t="s"><v>30</v></c><c r="B4" s="7" t="s"><v>31</v></c></row><row r="5" spans="1:2" x14ac:dyDescent="0.25"><c r="A5" s="7" t="s"><v>27</v></c><c r="B5" s="7" t="s"><v>0</v></c></row><row r="6" spans="1:2" x14ac:dyDescent="0.25"><c r="A6" s="7" t="s"><v>27</v></c><c r="B6" s="7" t="s"><v>1</v></c></row><row r="7" spans="1:2" x14ac:dyDescent="0.25"><c r="A7" s="7" t="s"><v>27</v></c><c r="B7" s="7" t="s"><v>2</v></c></row><row r="8" spans="1:2" x14ac:dyDescent="0.25"><c r="A8" s="7" t="s"><v>27</v></c><c r="B8" s="7" t="s"><v>3</v></c></row><row r="9" spans="1:2" x14ac:dyDescent="0.25"><c r="A9" s="7" t="s"><v>27</v></c><c r="B9" s="7" t="s"><v>6</v></c></row><row r="10" spans="1:2" x14ac:dyDescent="0.25"><c r="A10" s="7" t="s"><v>27</v></c><c r="B10" s="7" t="s"><v>7</v></c></row><row r="11" spans="1:2" x14ac:dyDescent="0.25"><c r="A11" s="7" t="s"><v>32</v></c><c r="B11" s="7" t="s"><v>33</v></c></row><row r="12" spans="1:2" x14ac:dyDescent="0.25"><c r="A12" s="7" t="s"><v>27</v></c><c r="B12" s="7" t="s"><v>4</v></c></row><row r="13" spans="1:2" x14ac:dyDescent="0.25"><c r="A13" s="7" t="s"><v>27</v></c><c r="B13" s="7" t="s"><v>5</v></c></row><row r="14" spans="1:2" x14ac:dyDescent="0.25"><c r="A14" s="7" t="s"><v>27</v></c><c r="B14" s="7" t="s"><v>8</v></c></row><row r="15" spans="1:2" x14ac:dyDescent="0.25"><c r="A15" s="7" t="s"><v>34</v></c><c r="B15" s="7" t="s"><v>35</v></c></row><row r="16" spans="1:2" x14ac:dyDescent="0.25"><c r="A16" s="7" t="s"><v>36</v></c><c r="B16" s="7" t="s"><v>37</v></c></row><row r="17" spans="1:2" x14ac:dyDescent="0.25"><c r="A17" s="7" t="s"><v>38</v></c><c r="B17" s="7" t="s"><v>39</v></c></row><row r="18" spans="1:2" x14ac:dyDescent="0.25"><c r="A18" s="7" t="s"><v>27</v></c><c r="B18" s="7" t="s"><v>40</v></c></row><row r="19" spans="1:2" x14ac:dyDescent="0.25"><c r="A19" s="7" t="s"><v>27</v></c><c r="B19" s="7" t="s"><v>41</v></c></row><row r="20" spans="1:2" x14ac:dyDescent="0.25"><c r="A20" s="7" t="s"><v>27</v></c><c r="B20" s="7" t="s"><v>42</v></c></row><row r="21" spans="1:2" x14ac:dyDescent="0.25"><c r="A21" s="7" t="s"><v>27</v></c><c r="B21" s="7" t="s"><v>43</v></c></row><row r="22" spans="1:2" x14ac:dyDescent="0.25"><c r="A22" s="7" t="s"><v>27</v></c><c r="B22" s="7" t="s"><v>44</v></c></row><row r="23" spans="1:2" x14ac:dyDescent="0.25"><c r="A23" s="7" t="s"><v>27</v></c><c r="B23" s="7" t="s"><v>45</v></c></row><row r="24" spans="1:2" x14ac:dyDescent="0.25"><c r="A24" s="7" t="s"><v>46</v></c><c r="B24" s="7" t="s"><v>47</v></c></row><row r="25" spans="1:2" x14ac:dyDescent="0.25"><c r="A25" s="7" t="s"><v>27</v></c><c r="B25" s="7" t="s"><v>11</v></c></row><row r="26" spans="1:2" x14ac:dyDescent="0.25"><c r="A26" s="7" t="s"><v>27</v></c><c r="B26" s="7" t="s"><v>48</v></c></row><row r="27" spans="1:2" x14ac:dyDescent="0.25"><c r="A27" s="7" t="s"><v>27</v></c><c r="B27" s="7" t="s"><v>19</v></c></row><row r="28" spans="1:2" x14ac:dyDescent="0.25"><c r="A28" s="7" t="s"><v>27</v></c><c r="B28" s="7" t="s"><v>49</v></c></row><row r="29" spans="1:2" x14ac:dyDescent="0.25"><c r="A29" s="7" t="s"><v>50</v></c><c r="B29" s="7" t="s"><v>51</v></c></row><row r="30" spans="1:2" x14ac:dyDescent="0.25"><c r="A30" s="7" t="s"><v>27</v></c><c r="B30" s="7" t="s"><v>52</v></c></row><row r="31" spans="1:2" x14ac:dyDescent="0.25"><c r="A31" s="7" t="s"><v>27</v></c><c r="B31" s="7" t="s"><v>53</v></c></row><row r="33" spans="1:2" x14ac:dyDescent="0.25"><c r="A33" s="7" t="s"><v>55</v></c><c r="B33" s="7" t="s"><v>56</v></c></row><row r="34" spans="1:2" x14ac:dyDescent="0.25"><c r="A34" s="7" t="s"><v>57</v></c><c r="B34" s="7" t="s"><v>58</v></c></row><row r="35" spans="1:2" x14ac:dyDescent="0.25"><c r="A35" s="7" t="s"><v>59</v></c><c r="B35" s="7" t="s"><v>60</v></c></row></sheetData><mergeCells count="2"><mergeCell ref="A1:B1"/><mergeCell ref="A2:B2"/></mergeCells><pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/></worksheet>
 </file>
</xml_diff>